<commit_message>
Add Memory Boost and Fem-Arosa photos to quotation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019b1TMg8cmtFFYPLUhebG5R
</commit_message>
<xml_diff>
--- a/product-data/quotation/Areej-Najd-Quotation.xlsx
+++ b/product-data/quotation/Areej-Najd-Quotation.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;_-* #,##0.00\-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="15">
     <font>
       <name val="Times New Roman"/>
       <charset val="204"/>
@@ -97,12 +97,6 @@
       <name val="Calibri"/>
       <color rgb="FF0000FF"/>
       <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="FF808080"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -248,7 +242,7 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -454,14 +448,11 @@
     <xf numFmtId="164" fontId="12" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -687,6 +678,56 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1009650" cy="1095375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="923925" cy="1095375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1317,11 +1358,7 @@
       <c r="G25" s="68" t="n">
         <v>15</v>
       </c>
-      <c r="H25" s="69" t="inlineStr">
-        <is>
-          <t>صورة غير متوفرة</t>
-        </is>
-      </c>
+      <c r="H25" s="64" t="n"/>
     </row>
     <row r="26" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A26" s="62" t="inlineStr">
@@ -1329,7 +1366,7 @@
           <t>762497361537</t>
         </is>
       </c>
-      <c r="B26" s="70" t="inlineStr"/>
+      <c r="B26" s="69" t="inlineStr"/>
       <c r="C26" s="64" t="inlineStr">
         <is>
           <t>Dr. Organic Fem-Arosa Drops 30 ml</t>
@@ -1346,11 +1383,7 @@
       <c r="G26" s="68" t="n">
         <v>12</v>
       </c>
-      <c r="H26" s="69" t="inlineStr">
-        <is>
-          <t>صورة غير متوفرة</t>
-        </is>
-      </c>
+      <c r="H26" s="64" t="n"/>
     </row>
     <row r="27" ht="17.4" customFormat="1" customHeight="1" s="19"/>
     <row r="28" ht="17.4" customFormat="1" customHeight="1" s="19"/>
@@ -1535,63 +1568,63 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="71" t="inlineStr">
+      <c r="A1" s="70" t="inlineStr">
         <is>
           <t>تعليمات تعبئة عرض السعر</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="72" t="inlineStr">
+      <c r="A2" s="71" t="inlineStr">
         <is>
           <t>الخلايا الصفراء في شيت Quotation محتاجة تتعبى قبل الإرسال:</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="72" t="inlineStr">
+      <c r="A3" s="71" t="inlineStr">
         <is>
           <t>• رقم العرض (QUOTE #) في G5، واسم اللي جهز العرض والإيميل في A10 و A11.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="72" t="inlineStr">
+      <c r="A4" s="71" t="inlineStr">
         <is>
           <t>• بيانات الشركة المرسل لها (A13 إلى A18): متسابة فاضية زي ما طلبت.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="72" t="inlineStr">
+      <c r="A5" s="71" t="inlineStr">
         <is>
           <t>• سعر البيع المقترح قبل الضريبة (العمود F). سعر البيع شامل الضريبة (العمود D) بيتحسب لوحده.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="72" t="inlineStr">
+      <c r="A6" s="71" t="inlineStr">
         <is>
           <t>• رقم تسجيل SFDA لفيم أروزا (B26): مش موجود في الملفات.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="72" t="inlineStr">
+      <c r="A7" s="71" t="inlineStr">
         <is>
           <t>• مدة السداد ومدة صلاحية العرض (A43 و A45)، واسم الموقّع (A49).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="72" t="inlineStr">
+      <c r="A8" s="71" t="inlineStr">
         <is>
           <t>الأرقام باللون الأزرق (سعر التوريد) منقولة من فاتورة رقم 54 بتاريخ 2026-10-01.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="72" t="inlineStr">
+      <c r="A9" s="71" t="inlineStr">
         <is>
           <t>مثال: لو سعر البيع المقترح 25 ريال قبل الضريبة، اكتب 25 في F والعمود D هيطلع 28.75.</t>
         </is>

</xml_diff>

<commit_message>
Quotation: replace supply price with recommended sales prices, white-background product photos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019b1TMg8cmtFFYPLUhebG5R
</commit_message>
<xml_diff>
--- a/product-data/quotation/Areej-Najd-Quotation.xlsx
+++ b/product-data/quotation/Areej-Najd-Quotation.xlsx
@@ -10,7 +10,7 @@
     <sheet name="تعليمات" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quotation'!$A$1:$H$56</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quotation'!$A$1:$G$56</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -242,7 +242,7 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -442,10 +442,7 @@
     <xf numFmtId="9" fontId="10" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="10" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="4" fontId="12" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -542,9 +539,9 @@
         <t>Rows 1-4: internal item codes from the invoice (no EAN barcode in the files).</t>
       </text>
     </comment>
-    <comment ref="G21" authorId="0" shapeId="0">
+    <comment ref="F21" authorId="0" shapeId="0">
       <text>
-        <t>Invoice prices (SAR, excl. VAT) taken from Areej Najd tax invoice No. 54 dated 2026-10-01.</t>
+        <t>Recommended public prices (SAR, before VAT) from the Dairy Mind distribution feasibility study, dated 29/09/2026.</t>
       </text>
     </comment>
     <comment ref="A26" authorId="0" shapeId="0">
@@ -590,12 +587,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
-      <colOff>0</colOff>
+      <col>6</col>
+      <colOff>247650</colOff>
       <row>20</row>
-      <rowOff>0</rowOff>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="1123950" cy="1095375"/>
+    <ext cx="1123950" cy="1123950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -615,12 +612,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
-      <colOff>0</colOff>
+      <col>6</col>
+      <colOff>247650</colOff>
       <row>21</row>
-      <rowOff>0</rowOff>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="1133475" cy="1095375"/>
+    <ext cx="1123950" cy="1123950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -640,12 +637,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
-      <colOff>0</colOff>
+      <col>6</col>
+      <colOff>247650</colOff>
       <row>22</row>
-      <rowOff>0</rowOff>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="1381125" cy="1095375"/>
+    <ext cx="1123950" cy="1123950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -665,12 +662,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
-      <colOff>0</colOff>
+      <col>6</col>
+      <colOff>247650</colOff>
       <row>23</row>
-      <rowOff>0</rowOff>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="923925" cy="1095375"/>
+    <ext cx="1123950" cy="1123950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -690,12 +687,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
-      <colOff>0</colOff>
+      <col>6</col>
+      <colOff>247650</colOff>
       <row>24</row>
-      <rowOff>0</rowOff>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="1009650" cy="1095375"/>
+    <ext cx="1123950" cy="1123950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -715,12 +712,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
-      <colOff>0</colOff>
+      <col>6</col>
+      <colOff>247650</colOff>
       <row>25</row>
-      <rowOff>0</rowOff>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="923925" cy="1095375"/>
+    <ext cx="1123950" cy="1123950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -1017,8 +1014,8 @@
     <col width="23.77734375" customWidth="1" style="54" min="4" max="4"/>
     <col width="18.33203125" bestFit="1" customWidth="1" style="7" min="5" max="5"/>
     <col width="18.33203125" customWidth="1" style="7" min="6" max="6"/>
-    <col width="21.77734375" bestFit="1" customWidth="1" style="7" min="7" max="7"/>
-    <col width="24" bestFit="1" customWidth="1" style="7" min="8" max="9"/>
+    <col width="24" bestFit="1" customWidth="1" style="7" min="7" max="7"/>
+    <col width="11.6640625" bestFit="1" customWidth="1" style="7" min="8" max="9"/>
     <col width="8.77734375" customWidth="1" style="7" min="10" max="10"/>
     <col width="19.77734375" bestFit="1" customWidth="1" style="7" min="11" max="11"/>
     <col width="8.77734375" customWidth="1" style="7" min="12" max="16384"/>
@@ -1205,11 +1202,6 @@
       </c>
       <c r="G20" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Invoice Price سعر التوريد </t>
-        </is>
-      </c>
-      <c r="H20" s="24" t="inlineStr">
-        <is>
           <t>Product Image
 صورة المنتج</t>
         </is>
@@ -1238,11 +1230,10 @@
       <c r="E21" s="66" t="n">
         <v>0.15</v>
       </c>
-      <c r="F21" s="67" t="n"/>
-      <c r="G21" s="68" t="n">
-        <v>11</v>
-      </c>
-      <c r="H21" s="64" t="n"/>
+      <c r="F21" s="67" t="n">
+        <v>65</v>
+      </c>
+      <c r="G21" s="64" t="n"/>
     </row>
     <row r="22" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A22" s="62" t="inlineStr">
@@ -1267,11 +1258,10 @@
       <c r="E22" s="66" t="n">
         <v>0.15</v>
       </c>
-      <c r="F22" s="67" t="n"/>
-      <c r="G22" s="68" t="n">
-        <v>8</v>
-      </c>
-      <c r="H22" s="64" t="n"/>
+      <c r="F22" s="67" t="n">
+        <v>55</v>
+      </c>
+      <c r="G22" s="64" t="n"/>
     </row>
     <row r="23" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A23" s="62" t="inlineStr">
@@ -1296,11 +1286,10 @@
       <c r="E23" s="66" t="n">
         <v>0.15</v>
       </c>
-      <c r="F23" s="67" t="n"/>
-      <c r="G23" s="68" t="n">
-        <v>6</v>
-      </c>
-      <c r="H23" s="64" t="n"/>
+      <c r="F23" s="67" t="n">
+        <v>30</v>
+      </c>
+      <c r="G23" s="64" t="n"/>
     </row>
     <row r="24" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A24" s="62" t="inlineStr">
@@ -1325,11 +1314,10 @@
       <c r="E24" s="66" t="n">
         <v>0.15</v>
       </c>
-      <c r="F24" s="67" t="n"/>
-      <c r="G24" s="68" t="n">
-        <v>7</v>
-      </c>
-      <c r="H24" s="64" t="n"/>
+      <c r="F24" s="67" t="n">
+        <v>55</v>
+      </c>
+      <c r="G24" s="64" t="n"/>
     </row>
     <row r="25" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A25" s="62" t="inlineStr">
@@ -1354,11 +1342,10 @@
       <c r="E25" s="66" t="n">
         <v>0.15</v>
       </c>
-      <c r="F25" s="67" t="n"/>
-      <c r="G25" s="68" t="n">
-        <v>15</v>
-      </c>
-      <c r="H25" s="64" t="n"/>
+      <c r="F25" s="67" t="n">
+        <v>156</v>
+      </c>
+      <c r="G25" s="64" t="n"/>
     </row>
     <row r="26" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A26" s="62" t="inlineStr">
@@ -1366,7 +1353,7 @@
           <t>762497361537</t>
         </is>
       </c>
-      <c r="B26" s="69" t="inlineStr"/>
+      <c r="B26" s="68" t="inlineStr"/>
       <c r="C26" s="64" t="inlineStr">
         <is>
           <t>Dr. Organic Fem-Arosa Drops 30 ml</t>
@@ -1379,11 +1366,10 @@
       <c r="E26" s="66" t="n">
         <v>0.15</v>
       </c>
-      <c r="F26" s="67" t="n"/>
-      <c r="G26" s="68" t="n">
-        <v>12</v>
-      </c>
-      <c r="H26" s="64" t="n"/>
+      <c r="F26" s="67" t="n">
+        <v>49</v>
+      </c>
+      <c r="G26" s="64" t="n"/>
     </row>
     <row r="27" ht="17.4" customFormat="1" customHeight="1" s="19"/>
     <row r="28" ht="17.4" customFormat="1" customHeight="1" s="19"/>
@@ -1480,7 +1466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>3. All prices are in Saudi Riyal (SAR). Invoice price excludes 15% VAT</t>
+          <t>3. All prices are in Saudi Riyal (SAR). Recommended sales price excludes 15% VAT</t>
         </is>
       </c>
       <c r="E44" s="8" t="n"/>
@@ -1568,65 +1554,65 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="70" t="inlineStr">
+      <c r="A1" s="69" t="inlineStr">
         <is>
           <t>تعليمات تعبئة عرض السعر</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="71" t="inlineStr">
+      <c r="A2" s="70" t="inlineStr">
         <is>
           <t>الخلايا الصفراء في شيت Quotation محتاجة تتعبى قبل الإرسال:</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="71" t="inlineStr">
+      <c r="A3" s="70" t="inlineStr">
         <is>
           <t>• رقم العرض (QUOTE #) في G5، واسم اللي جهز العرض والإيميل في A10 و A11.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="71" t="inlineStr">
+      <c r="A4" s="70" t="inlineStr">
         <is>
           <t>• بيانات الشركة المرسل لها (A13 إلى A18): متسابة فاضية زي ما طلبت.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="71" t="inlineStr">
-        <is>
-          <t>• سعر البيع المقترح قبل الضريبة (العمود F). سعر البيع شامل الضريبة (العمود D) بيتحسب لوحده.</t>
+      <c r="A5" s="70" t="inlineStr">
+        <is>
+          <t>• سعر البيع المقترح قبل الضريبة (العمود F) منقول من دراسة الجدوى. سعر البيع شامل الضريبة (العمود D) بيتحسب لوحده.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="71" t="inlineStr">
+      <c r="A6" s="70" t="inlineStr">
         <is>
           <t>• رقم تسجيل SFDA لفيم أروزا (B26): مش موجود في الملفات.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="71" t="inlineStr">
+      <c r="A7" s="70" t="inlineStr">
         <is>
           <t>• مدة السداد ومدة صلاحية العرض (A43 و A45)، واسم الموقّع (A49).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="71" t="inlineStr">
-        <is>
-          <t>الأرقام باللون الأزرق (سعر التوريد) منقولة من فاتورة رقم 54 بتاريخ 2026-10-01.</t>
+      <c r="A8" s="70" t="inlineStr">
+        <is>
+          <t>الأرقام باللون الأزرق (سعر البيع المقترح) منقولة من دراسة جدوى ديير مايند بتاريخ 29/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="71" t="inlineStr">
-        <is>
-          <t>مثال: لو سعر البيع المقترح 25 ريال قبل الضريبة، اكتب 25 في F والعمود D هيطلع 28.75.</t>
+      <c r="A9" s="70" t="inlineStr">
+        <is>
+          <t>مثال: سعر البيع المقترح 65 ريال قبل الضريبة في F، والعمود D بيطلع 74.75.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Fem-Arosa SFDA registration number to quotation and product sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019b1TMg8cmtFFYPLUhebG5R
</commit_message>
<xml_diff>
--- a/product-data/quotation/Areej-Najd-Quotation.xlsx
+++ b/product-data/quotation/Areej-Najd-Quotation.xlsx
@@ -242,7 +242,7 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -443,9 +443,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="12" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -551,7 +548,7 @@
     </comment>
     <comment ref="B26" authorId="0" shapeId="0">
       <text>
-        <t>No final SFDA product number in the files received (registration request view 1039643). Fill in before sending.</t>
+        <t>SFDA registration number from the Ghad platform screenshot sent by the user (barcode 00762497361537).</t>
       </text>
     </comment>
   </commentList>
@@ -1353,7 +1350,11 @@
           <t>762497361537</t>
         </is>
       </c>
-      <c r="B26" s="68" t="inlineStr"/>
+      <c r="B26" s="63" t="inlineStr">
+        <is>
+          <t>FOM-24-56091-FOP-110126-10077-C-12688-5160</t>
+        </is>
+      </c>
       <c r="C26" s="64" t="inlineStr">
         <is>
           <t>Dr. Organic Fem-Arosa Drops 30 ml</t>
@@ -1547,70 +1548,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="69" t="inlineStr">
+      <c r="A1" s="68" t="inlineStr">
         <is>
           <t>تعليمات تعبئة عرض السعر</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="70" t="inlineStr">
+      <c r="A2" s="69" t="inlineStr">
         <is>
           <t>الخلايا الصفراء في شيت Quotation محتاجة تتعبى قبل الإرسال:</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="70" t="inlineStr">
+      <c r="A3" s="69" t="inlineStr">
         <is>
           <t>• رقم العرض (QUOTE #) في G5، واسم اللي جهز العرض والإيميل في A10 و A11.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="70" t="inlineStr">
+      <c r="A4" s="69" t="inlineStr">
         <is>
           <t>• بيانات الشركة المرسل لها (A13 إلى A18): متسابة فاضية زي ما طلبت.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="70" t="inlineStr">
+      <c r="A5" s="69" t="inlineStr">
         <is>
           <t>• سعر البيع المقترح قبل الضريبة (العمود F) منقول من دراسة الجدوى. سعر البيع شامل الضريبة (العمود D) بيتحسب لوحده.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="70" t="inlineStr">
-        <is>
-          <t>• رقم تسجيل SFDA لفيم أروزا (B26): مش موجود في الملفات.</t>
+      <c r="A6" s="69" t="inlineStr">
+        <is>
+          <t>• مدة السداد ومدة صلاحية العرض (A43 و A45)، واسم الموقّع (A49).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="70" t="inlineStr">
-        <is>
-          <t>• مدة السداد ومدة صلاحية العرض (A43 و A45)، واسم الموقّع (A49).</t>
+      <c r="A7" s="69" t="inlineStr">
+        <is>
+          <t>الأرقام باللون الأزرق (سعر البيع المقترح) منقولة من دراسة جدوى ديير مايند بتاريخ 29/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="70" t="inlineStr">
-        <is>
-          <t>الأرقام باللون الأزرق (سعر البيع المقترح) منقولة من دراسة جدوى ديير مايند بتاريخ 29/09/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="70" t="inlineStr">
+      <c r="A8" s="69" t="inlineStr">
         <is>
           <t>مثال: سعر البيع المقترح 65 ريال قبل الضريبة في F، والعمود D بيطلع 74.75.</t>
         </is>

</xml_diff>

<commit_message>
Quotation: list Memory Boost and Fem-Arosa first
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019b1TMg8cmtFFYPLUhebG5R
</commit_message>
<xml_diff>
--- a/product-data/quotation/Areej-Najd-Quotation.xlsx
+++ b/product-data/quotation/Areej-Najd-Quotation.xlsx
@@ -531,24 +531,24 @@
     <author>Quotation</author>
   </authors>
   <commentList>
-    <comment ref="A21" authorId="0" shapeId="0">
-      <text>
-        <t>Rows 1-4: internal item codes from the invoice (no EAN barcode in the files).</t>
-      </text>
-    </comment>
     <comment ref="F21" authorId="0" shapeId="0">
       <text>
         <t>Recommended public prices (SAR, before VAT) from the Dairy Mind distribution feasibility study, dated 29/09/2026.</t>
       </text>
     </comment>
-    <comment ref="A26" authorId="0" shapeId="0">
+    <comment ref="A22" authorId="0" shapeId="0">
       <text>
         <t>Barcode from the SFDA food-product registration record (00762497361537). Invoice internal code: 10108.</t>
       </text>
     </comment>
-    <comment ref="B26" authorId="0" shapeId="0">
+    <comment ref="B22" authorId="0" shapeId="0">
       <text>
         <t>SFDA registration number from the Ghad platform screenshot sent by the user (barcode 00762497361537).</t>
+      </text>
+    </comment>
+    <comment ref="A23" authorId="0" shapeId="0">
+      <text>
+        <t>Rows 3-6: internal item codes from the invoice (no EAN barcode in the files).</t>
       </text>
     </comment>
   </commentList>
@@ -1207,17 +1207,17 @@
     <row r="21" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A21" s="62" t="inlineStr">
         <is>
-          <t>10044</t>
+          <t>762497361506</t>
         </is>
       </c>
       <c r="B21" s="63" t="inlineStr">
         <is>
-          <t>CN-2023-36519</t>
+          <t>FOP-251125-1028812</t>
         </is>
       </c>
       <c r="C21" s="64" t="inlineStr">
         <is>
-          <t>Femina Vaginal Foam – Feminine Hygiene Foaming Cleanser 200 ml</t>
+          <t>Dr. Organic Memory Boost Syrup 120 ml</t>
         </is>
       </c>
       <c r="D21" s="65">
@@ -1228,24 +1228,24 @@
         <v>0.15</v>
       </c>
       <c r="F21" s="67" t="n">
-        <v>65</v>
+        <v>156</v>
       </c>
       <c r="G21" s="64" t="n"/>
     </row>
     <row r="22" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A22" s="62" t="inlineStr">
         <is>
-          <t>10063</t>
+          <t>762497361537</t>
         </is>
       </c>
       <c r="B22" s="63" t="inlineStr">
         <is>
-          <t>CN-2023-84129</t>
+          <t>FOM-24-56091-FOP-110126-10077-C-12688-5160</t>
         </is>
       </c>
       <c r="C22" s="64" t="inlineStr">
         <is>
-          <t>Aviance Octo Anti-Dandruff Shampoo 200 ml</t>
+          <t>Dr. Organic Fem-Arosa Drops 30 ml</t>
         </is>
       </c>
       <c r="D22" s="65">
@@ -1256,24 +1256,24 @@
         <v>0.15</v>
       </c>
       <c r="F22" s="67" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G22" s="64" t="n"/>
     </row>
     <row r="23" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A23" s="62" t="inlineStr">
         <is>
-          <t>10001</t>
+          <t>10044</t>
         </is>
       </c>
       <c r="B23" s="63" t="inlineStr">
         <is>
-          <t>CN-2026-65086</t>
+          <t>CN-2023-36519</t>
         </is>
       </c>
       <c r="C23" s="64" t="inlineStr">
         <is>
-          <t>E-Panthen Moisturizing Cream (5% D-Panthenol + Vit E)</t>
+          <t>Femina Vaginal Foam – Feminine Hygiene Foaming Cleanser 200 ml</t>
         </is>
       </c>
       <c r="D23" s="65">
@@ -1284,24 +1284,24 @@
         <v>0.15</v>
       </c>
       <c r="F23" s="67" t="n">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="G23" s="64" t="n"/>
     </row>
     <row r="24" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A24" s="62" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>10063</t>
         </is>
       </c>
       <c r="B24" s="63" t="inlineStr">
         <is>
-          <t>CN-2026-65103</t>
+          <t>CN-2023-84129</t>
         </is>
       </c>
       <c r="C24" s="64" t="inlineStr">
         <is>
-          <t>Mebonol Healing Cream</t>
+          <t>Aviance Octo Anti-Dandruff Shampoo 200 ml</t>
         </is>
       </c>
       <c r="D24" s="65">
@@ -1319,17 +1319,17 @@
     <row r="25" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A25" s="62" t="inlineStr">
         <is>
-          <t>762497361506</t>
+          <t>10001</t>
         </is>
       </c>
       <c r="B25" s="63" t="inlineStr">
         <is>
-          <t>FOP-251125-1028812</t>
+          <t>CN-2026-65086</t>
         </is>
       </c>
       <c r="C25" s="64" t="inlineStr">
         <is>
-          <t>Dr. Organic Memory Boost Syrup 120 ml</t>
+          <t>E-Panthen Moisturizing Cream (5% D-Panthenol + Vit E)</t>
         </is>
       </c>
       <c r="D25" s="65">
@@ -1340,24 +1340,24 @@
         <v>0.15</v>
       </c>
       <c r="F25" s="67" t="n">
-        <v>156</v>
+        <v>30</v>
       </c>
       <c r="G25" s="64" t="n"/>
     </row>
     <row r="26" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A26" s="62" t="inlineStr">
         <is>
-          <t>762497361537</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="B26" s="63" t="inlineStr">
         <is>
-          <t>FOM-24-56091-FOP-110126-10077-C-12688-5160</t>
+          <t>CN-2026-65103</t>
         </is>
       </c>
       <c r="C26" s="64" t="inlineStr">
         <is>
-          <t>Dr. Organic Fem-Arosa Drops 30 ml</t>
+          <t>Mebonol Healing Cream</t>
         </is>
       </c>
       <c r="D26" s="65">
@@ -1368,7 +1368,7 @@
         <v>0.15</v>
       </c>
       <c r="F26" s="67" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="G26" s="64" t="n"/>
     </row>

</xml_diff>

<commit_message>
Quotation: remove mobile number and leftover template fax
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019b1TMg8cmtFFYPLUhebG5R
</commit_message>
<xml_diff>
--- a/product-data/quotation/Areej-Najd-Quotation.xlsx
+++ b/product-data/quotation/Areej-Najd-Quotation.xlsx
@@ -1082,11 +1082,7 @@
       <c r="C8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Mobile: 0504152111</t>
-        </is>
-      </c>
+      <c r="A9" s="6" t="n"/>
       <c r="C9" s="8" t="n"/>
     </row>
     <row r="10">
@@ -1518,7 +1514,7 @@
     <row r="54">
       <c r="A54" s="54" t="inlineStr">
         <is>
-          <t>[ Areej Najd Est. , Mobile: 0504152111 , Riyadh ]</t>
+          <t>[ Areej Najd Est. , Riyadh ]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update SFDA registration numbers and barcodes from official records
Memory Boost and Sleep full registration numbers; barcodes for all
six quoted products; Femina/Octo/E-Panthen/Mebonol notification details.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019b1TMg8cmtFFYPLUhebG5R
</commit_message>
<xml_diff>
--- a/product-data/quotation/Areej-Najd-Quotation.xlsx
+++ b/product-data/quotation/Areej-Najd-Quotation.xlsx
@@ -538,17 +538,12 @@
     </comment>
     <comment ref="A22" authorId="0" shapeId="0">
       <text>
-        <t>Barcode from the SFDA food-product registration record (00762497361537). Invoice internal code: 10108.</t>
+        <t>All barcodes as listed on the SFDA registration/notification records (verified by the user).</t>
       </text>
     </comment>
     <comment ref="B22" authorId="0" shapeId="0">
       <text>
         <t>SFDA registration number from the Ghad platform screenshot sent by the user (barcode 00762497361537).</t>
-      </text>
-    </comment>
-    <comment ref="A23" authorId="0" shapeId="0">
-      <text>
-        <t>Rows 3-6: internal item codes from the invoice (no EAN barcode in the files).</t>
       </text>
     </comment>
   </commentList>
@@ -1203,12 +1198,12 @@
     <row r="21" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A21" s="62" t="inlineStr">
         <is>
-          <t>762497361506</t>
+          <t>00762497361506</t>
         </is>
       </c>
       <c r="B21" s="63" t="inlineStr">
         <is>
-          <t>FOP-251125-1028812</t>
+          <t>FOM-24-272344-FOP-251125-1028812-C-12688-881856</t>
         </is>
       </c>
       <c r="C21" s="64" t="inlineStr">
@@ -1231,7 +1226,7 @@
     <row r="22" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A22" s="62" t="inlineStr">
         <is>
-          <t>762497361537</t>
+          <t>00762497361537</t>
         </is>
       </c>
       <c r="B22" s="63" t="inlineStr">
@@ -1259,7 +1254,7 @@
     <row r="23" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A23" s="62" t="inlineStr">
         <is>
-          <t>10044</t>
+          <t>6772505023146</t>
         </is>
       </c>
       <c r="B23" s="63" t="inlineStr">
@@ -1287,7 +1282,7 @@
     <row r="24" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A24" s="62" t="inlineStr">
         <is>
-          <t>10063</t>
+          <t>6772505023108</t>
         </is>
       </c>
       <c r="B24" s="63" t="inlineStr">
@@ -1315,7 +1310,7 @@
     <row r="25" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A25" s="62" t="inlineStr">
         <is>
-          <t>10001</t>
+          <t>6224010064195</t>
         </is>
       </c>
       <c r="B25" s="63" t="inlineStr">
@@ -1325,7 +1320,7 @@
       </c>
       <c r="C25" s="64" t="inlineStr">
         <is>
-          <t>E-Panthen Moisturizing Cream (5% D-Panthenol + Vit E)</t>
+          <t>E-Panthen Moisturizing Cream (5% D-Panthenol + Vit E) 40 g</t>
         </is>
       </c>
       <c r="D25" s="65">
@@ -1343,7 +1338,7 @@
     <row r="26" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A26" s="62" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>6224010064188</t>
         </is>
       </c>
       <c r="B26" s="63" t="inlineStr">
@@ -1353,7 +1348,7 @@
       </c>
       <c r="C26" s="64" t="inlineStr">
         <is>
-          <t>Mebonol Healing Cream</t>
+          <t>Mebonol Healing Cream 40 g</t>
         </is>
       </c>
       <c r="D26" s="65">

</xml_diff>